<commit_message>
scan: seg4 2026-08-10 15:53 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq5_2026-08-10.xlsx
+++ b/output/full_scan/batch_seq5_2026-08-10.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O72"/>
+  <dimension ref="A1:O91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -845,38 +845,38 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>6112</v>
+        <v>4987</v>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>邁達特</t>
+          <t>科誠</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
         <v/>
       </c>
       <c r="D8" s="2" t="n">
-        <v>576.1866980412543</v>
+        <v>584.8800228060518</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>46.65</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="G8" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>66.69017822517257</v>
+        <v>55.06266666972992</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>33.93433000454363</v>
+        <v>23.90740117852677</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>1.557130807751481</v>
+        <v>0.750864911342356</v>
       </c>
       <c r="K8" s="2" t="n">
         <v>0</v>
@@ -888,31 +888,31 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>0.8764142552910098</v>
+        <v>-0.040881259379903</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>volume_break, rsi_strong, breakout_20d, market_above_ma60, adx_trending, obv_uptrend, breakout_volume_confirm, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>4938</v>
+        <v>4995</v>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>和碩</t>
+          <t>晶達</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
         <v/>
       </c>
       <c r="D9" s="2" t="n">
-        <v>565.2093206341074</v>
+        <v>581.8834410089281</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>89.5</v>
+        <v>49.65</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
@@ -923,13 +923,13 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>58.7542331573278</v>
+        <v>61.89391107408326</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>13.00077396795245</v>
+        <v>21.89643128718104</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>0.5340050343295596</v>
+        <v>0.3680819265057368</v>
       </c>
       <c r="K9" s="2" t="n">
         <v>0</v>
@@ -941,31 +941,31 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>0.5815481491111673</v>
+        <v>0.1877949283011947</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, adx_trending, obv_uptrend, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>5469</v>
+        <v>6112</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>瀚宇博</t>
+          <t>邁達特</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
         <v/>
       </c>
       <c r="D10" s="2" t="n">
-        <v>502.4246598896054</v>
+        <v>576.1866980412543</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>75.90000000000001</v>
+        <v>46.65</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
@@ -976,13 +976,13 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>54.84207341538713</v>
+        <v>66.69017822517257</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>31.38338938765148</v>
+        <v>33.93433000454363</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>1.675395321946261</v>
+        <v>1.557130807751481</v>
       </c>
       <c r="K10" s="2" t="n">
         <v>0</v>
@@ -994,31 +994,31 @@
         <v>-1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>1.12707051055253</v>
+        <v>0.8764142552910098</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, cci_momentum, mfi_strong</t>
+          <t>volume_break, rsi_strong, breakout_20d, market_above_ma60, adx_trending, obv_uptrend, breakout_volume_confirm, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>5471</v>
+        <v>4971</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>松翰</t>
+          <t>IET-KY</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
         <v/>
       </c>
       <c r="D11" s="2" t="n">
-        <v>493.0832019714096</v>
+        <v>574.9324408620763</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>56.7</v>
+        <v>502</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
@@ -1029,13 +1029,13 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>52.30787867763566</v>
+        <v>58.34648732163721</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>21.54622246994404</v>
+        <v>25.97684300575536</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>1.078509125397793</v>
+        <v>2.135221367474606</v>
       </c>
       <c r="K11" s="2" t="n">
         <v>0</v>
@@ -1047,31 +1047,31 @@
         <v>-1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>0.2958015930794606</v>
+        <v>19.98532867420871</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>volume_break, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, breakout_volume_confirm, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>4976</v>
+        <v>4938</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>佳凌</t>
+          <t>和碩</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
         <v/>
       </c>
       <c r="D12" s="2" t="n">
-        <v>482.5901690836005</v>
+        <v>565.2093206341074</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>36.15</v>
+        <v>89.5</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
@@ -1082,13 +1082,13 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>51.26779169239151</v>
+        <v>58.7542331573278</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>27.86231293698093</v>
+        <v>13.00077396795245</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>0.2829372028090996</v>
+        <v>0.5340050343295596</v>
       </c>
       <c r="K12" s="2" t="n">
         <v>0</v>
@@ -1100,31 +1100,31 @@
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>0.2575622567812074</v>
+        <v>0.5815481491111673</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>6142</v>
+        <v>4931</v>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>友勁</t>
+          <t>新盛力</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
         <v/>
       </c>
       <c r="D13" s="2" t="n">
-        <v>456.1158941779074</v>
+        <v>560.9245463978301</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>9.630000000000001</v>
+        <v>238</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
@@ -1135,16 +1135,16 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>49.98438217689223</v>
+        <v>59.30738278367268</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>26.47870798293671</v>
+        <v>23.70748922893275</v>
       </c>
       <c r="J13" s="2" t="n">
-        <v>0.3359395338855382</v>
+        <v>0.6558760169727845</v>
       </c>
       <c r="K13" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L13" s="2" t="n">
         <v>0</v>
@@ -1153,31 +1153,31 @@
         <v>-1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>-0.0551673406317408</v>
+        <v>5.274674958745038</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, adx_trending, cci_momentum, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>4903</v>
+        <v>5469</v>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>聯光通</t>
+          <t>瀚宇博</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
         <v/>
       </c>
       <c r="D14" s="2" t="n">
-        <v>454.0033093479357</v>
+        <v>502.4246598896054</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>41.8</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
@@ -1188,16 +1188,16 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>57.8043304416859</v>
+        <v>54.84207341538713</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>13.55416265088198</v>
+        <v>31.38338938765148</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>1.224716402546831</v>
+        <v>1.675395321946261</v>
       </c>
       <c r="K14" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L14" s="2" t="n">
         <v>0</v>
@@ -1206,31 +1206,31 @@
         <v>-1</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>0.6721449988859457</v>
+        <v>1.12707051055253</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, obv_uptrend, cci_momentum, mfi_strong</t>
+          <t>volume_break, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, cci_momentum, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>6153</v>
+        <v>5471</v>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>嘉聯益</t>
+          <t>松翰</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
         <v/>
       </c>
       <c r="D15" s="2" t="n">
-        <v>452.5795520264314</v>
+        <v>493.0832019714096</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>16.6</v>
+        <v>56.7</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1241,13 +1241,13 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46.84749936842287</v>
+        <v>52.30787867763566</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>38.11698692392985</v>
+        <v>21.54622246994404</v>
       </c>
       <c r="J15" s="2" t="n">
-        <v>0.6106620197777461</v>
+        <v>1.078509125397793</v>
       </c>
       <c r="K15" s="2" t="n">
         <v>0</v>
@@ -1259,31 +1259,31 @@
         <v>-1</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>0.2623625540956396</v>
+        <v>0.2958015930794606</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>4999</v>
+        <v>4939</v>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>鑫禾</t>
+          <t>亞電</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
         <v/>
       </c>
       <c r="D16" s="2" t="n">
-        <v>440.1548756261138</v>
+        <v>490.5817639174526</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>19.3</v>
+        <v>61.3</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
@@ -1294,13 +1294,13 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>51.19800122471387</v>
+        <v>52.84019835080345</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>20.28089994681724</v>
+        <v>17.0532326856979</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>2.903572112996284</v>
+        <v>0.4825377912407168</v>
       </c>
       <c r="K16" s="2" t="n">
         <v>0</v>
@@ -1312,31 +1312,31 @@
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>0.0277140310930834</v>
+        <v>0.1792423374161565</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, volume_break, market_above_ma60, avoid_chase, hist_turn_positive, adx_trending, williams_r_recovery</t>
+          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, liquidity_ok, hist_turn_positive, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>6116</v>
+        <v>4973</v>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>彩晶</t>
+          <t>廣穎</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
         <v/>
       </c>
       <c r="D17" s="2" t="n">
-        <v>434.7108060148295</v>
+        <v>487.5667747629464</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>14.9</v>
+        <v>162</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
@@ -1347,13 +1347,13 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>52.40162258130672</v>
+        <v>57.31033509986784</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>30.93984614256375</v>
+        <v>19.03912778809711</v>
       </c>
       <c r="J17" s="2" t="n">
-        <v>2.037502805417353</v>
+        <v>1.786535492428398</v>
       </c>
       <c r="K17" s="2" t="n">
         <v>0</v>
@@ -1365,31 +1365,31 @@
         <v>-1</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>0.1977560502766815</v>
+        <v>3.702204655989748</v>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, liquidity_ok, adx_trending, mfi_strong</t>
+          <t>ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>4919</v>
+        <v>4976</v>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>新唐</t>
+          <t>佳凌</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
         <v/>
       </c>
       <c r="D18" s="2" t="n">
-        <v>429.3850293103224</v>
+        <v>482.5901690836005</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>127.5</v>
+        <v>36.15</v>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
@@ -1400,13 +1400,13 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>43.22866779591424</v>
+        <v>51.26779169239151</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>27.56790810900981</v>
+        <v>27.86231293698093</v>
       </c>
       <c r="J18" s="2" t="n">
-        <v>0.6341136507146627</v>
+        <v>0.2829372028090996</v>
       </c>
       <c r="K18" s="2" t="n">
         <v>0</v>
@@ -1418,31 +1418,31 @@
         <v>-1</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>1.196276669922692</v>
+        <v>0.2575622567812074</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>4915</v>
+        <v>4903</v>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>致伸</t>
+          <t>聯光通</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
         <v/>
       </c>
       <c r="D19" s="2" t="n">
-        <v>423.4368021810705</v>
+        <v>474.0033093479357</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>60.7</v>
+        <v>41.8</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
@@ -1453,16 +1453,16 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>33.00319615903442</v>
+        <v>57.8043304416859</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>36.51958127973563</v>
+        <v>13.55416265088198</v>
       </c>
       <c r="J19" s="2" t="n">
-        <v>0.6543104038395353</v>
+        <v>1.224716402546831</v>
       </c>
       <c r="K19" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L19" s="2" t="n">
         <v>0</v>
@@ -1471,31 +1471,31 @@
         <v>-1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>-0.2193485453564638</v>
+        <v>0.6721449988859457</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross</t>
+          <t>rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, obv_uptrend, cci_momentum, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>6108</v>
+        <v>6142</v>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>競國</t>
+          <t>友勁</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
         <v/>
       </c>
       <c r="D20" s="2" t="n">
-        <v>423.1025774546979</v>
+        <v>456.1158941779074</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>18.7</v>
+        <v>9.630000000000001</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
@@ -1506,13 +1506,13 @@
         <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>62.38269000549838</v>
+        <v>49.98438217689223</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>22.82672744613928</v>
+        <v>26.47870798293671</v>
       </c>
       <c r="J20" s="2" t="n">
-        <v>0.7554640803048447</v>
+        <v>0.3359395338855382</v>
       </c>
       <c r="K20" s="2" t="n">
         <v>0</v>
@@ -1524,31 +1524,31 @@
         <v>-1</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>0.3134070327403515</v>
+        <v>-0.0551673406317408</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>4989</v>
+        <v>4760</v>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>榮科</t>
+          <t>勤凱</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
         <v/>
       </c>
       <c r="D21" s="2" t="n">
-        <v>420.796966263721</v>
+        <v>454.7339939511766</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>67.5</v>
+        <v>245</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
@@ -1559,16 +1559,16 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>45.74132719956933</v>
+        <v>44.9023529440021</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>21.09729325469074</v>
+        <v>31.92870852496787</v>
       </c>
       <c r="J21" s="2" t="n">
-        <v>0.7300041645655347</v>
+        <v>0.4062209305870837</v>
       </c>
       <c r="K21" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L21" s="2" t="n">
         <v>0</v>
@@ -1577,31 +1577,31 @@
         <v>-1</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>1.293873700175427</v>
+        <v>5.558106703927017</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, kd_golden_cross, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, kd_golden_cross, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>5484</v>
+        <v>6153</v>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>慧友</t>
+          <t>嘉聯益</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
         <v/>
       </c>
       <c r="D22" s="2" t="n">
-        <v>415.6682510653362</v>
+        <v>452.5795520264314</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>45.35</v>
+        <v>16.6</v>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
@@ -1612,13 +1612,13 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>57.21859493360295</v>
+        <v>46.84749936842287</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>16.69842979840663</v>
+        <v>38.11698692392985</v>
       </c>
       <c r="J22" s="2" t="n">
-        <v>2.175273072939902</v>
+        <v>0.6106620197777461</v>
       </c>
       <c r="K22" s="2" t="n">
         <v>0</v>
@@ -1630,31 +1630,31 @@
         <v>-1</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>0.7378793611678285</v>
+        <v>0.2623625540956396</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>4760</v>
+        <v>4542</v>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>勤凱</t>
+          <t>科嶠</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
         <v/>
       </c>
       <c r="D23" s="2" t="n">
-        <v>414.7339939511766</v>
+        <v>451.8328743084249</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>245</v>
+        <v>292.5</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
@@ -1665,16 +1665,16 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>44.9023529440021</v>
+        <v>46.03857010876823</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>31.92870852496787</v>
+        <v>24.92549018168834</v>
       </c>
       <c r="J23" s="2" t="n">
-        <v>0.4062209305870837</v>
+        <v>0.9534901560208164</v>
       </c>
       <c r="K23" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L23" s="2" t="n">
         <v>0</v>
@@ -1683,31 +1683,31 @@
         <v>-1</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>5.558106703927017</v>
+        <v>1.455698511003472</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, kd_golden_cross, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>4542</v>
+        <v>4999</v>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>科嶠</t>
+          <t>鑫禾</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
         <v/>
       </c>
       <c r="D24" s="2" t="n">
-        <v>411.8328743084249</v>
+        <v>440.1548756261138</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>292.5</v>
+        <v>19.3</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
@@ -1718,13 +1718,13 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46.03857010876823</v>
+        <v>51.19800122471387</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>24.92549018168834</v>
+        <v>20.28089994681724</v>
       </c>
       <c r="J24" s="2" t="n">
-        <v>0.9534901560208164</v>
+        <v>2.903572112996284</v>
       </c>
       <c r="K24" s="2" t="n">
         <v>0</v>
@@ -1736,31 +1736,31 @@
         <v>-1</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>1.455698511003472</v>
+        <v>0.0277140310930834</v>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>macd_golden_cross, volume_break, market_above_ma60, avoid_chase, hist_turn_positive, adx_trending, williams_r_recovery</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>5236</v>
+        <v>6116</v>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>凌陽創新</t>
+          <t>彩晶</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
         <v/>
       </c>
       <c r="D25" s="2" t="n">
-        <v>386.1000720665844</v>
+        <v>434.7108060148295</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>144</v>
+        <v>14.9</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
@@ -1771,13 +1771,13 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>42.52985307112612</v>
+        <v>52.40162258130672</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>32.45358889146563</v>
+        <v>30.93984614256375</v>
       </c>
       <c r="J25" s="2" t="n">
-        <v>0.4931189176599256</v>
+        <v>2.037502805417353</v>
       </c>
       <c r="K25" s="2" t="n">
         <v>0</v>
@@ -1789,31 +1789,31 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>0.5890449523042527</v>
+        <v>0.1977560502766815</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, liquidity_ok, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>6155</v>
+        <v>4919</v>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>鈞寶</t>
+          <t>新唐</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
         <v/>
       </c>
       <c r="D26" s="2" t="n">
-        <v>372.4576796129931</v>
+        <v>429.3850293103224</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>53.2</v>
+        <v>127.5</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
@@ -1824,13 +1824,13 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>37.33131055854724</v>
+        <v>43.22866779591424</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>28.61686991395724</v>
+        <v>27.56790810900981</v>
       </c>
       <c r="J26" s="2" t="n">
-        <v>0.810221052209947</v>
+        <v>0.6341136507146627</v>
       </c>
       <c r="K26" s="2" t="n">
         <v>0</v>
@@ -1842,31 +1842,31 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>0.538740303179158</v>
+        <v>1.196276669922692</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>4952</v>
+        <v>4915</v>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>凌通</t>
+          <t>致伸</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
         <v/>
       </c>
       <c r="D27" s="2" t="n">
-        <v>370.8651139957474</v>
+        <v>423.4368021810705</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>49.7</v>
+        <v>60.7</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
@@ -1877,13 +1877,13 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>49.00483017465969</v>
+        <v>33.00319615903442</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>25.28937153556218</v>
+        <v>36.51958127973563</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>1.604152488571844</v>
+        <v>0.6543104038395353</v>
       </c>
       <c r="K27" s="2" t="n">
         <v>0</v>
@@ -1895,31 +1895,31 @@
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>0.4579933470581394</v>
+        <v>-0.2193485453564638</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>5215</v>
+        <v>6108</v>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>科嘉-KY</t>
+          <t>競國</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
         <v/>
       </c>
       <c r="D28" s="2" t="n">
-        <v>365.4361974913245</v>
+        <v>423.1025774546979</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>38.2</v>
+        <v>18.7</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
@@ -1930,13 +1930,13 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>38.65508097197239</v>
+        <v>62.38269000549838</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>27.13068633506663</v>
+        <v>22.82672744613928</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>0.2826567577724452</v>
+        <v>0.7554640803048447</v>
       </c>
       <c r="K28" s="2" t="n">
         <v>0</v>
@@ -1948,31 +1948,31 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>0.1298262283225051</v>
+        <v>0.3134070327403515</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>4949</v>
+        <v>4989</v>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>有成精密</t>
+          <t>榮科</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
         <v/>
       </c>
       <c r="D29" s="2" t="n">
-        <v>364.2997256912519</v>
+        <v>420.796966263721</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>72.5</v>
+        <v>67.5</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
@@ -1983,13 +1983,13 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>53.3543493247271</v>
+        <v>45.74132719956933</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>24.48047351854383</v>
+        <v>21.09729325469074</v>
       </c>
       <c r="J29" s="2" t="n">
-        <v>0.9126413295161788</v>
+        <v>0.7300041645655347</v>
       </c>
       <c r="K29" s="2" t="n">
         <v>0</v>
@@ -2001,31 +2001,31 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>1.483521275588549</v>
+        <v>1.293873700175427</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, kd_golden_cross, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>4912</v>
+        <v>4951</v>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>聯德控股-KY</t>
+          <t>精拓科</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
         <v/>
       </c>
       <c r="D30" s="2" t="n">
-        <v>363.2468637203646</v>
+        <v>417.0485411398608</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>89.8</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
@@ -2036,16 +2036,16 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>56.31566008128947</v>
+        <v>40.65317999530525</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>19.52800831960572</v>
+        <v>33.39051182545554</v>
       </c>
       <c r="J30" s="2" t="n">
-        <v>1.453387628466162</v>
+        <v>0.6558288277315413</v>
       </c>
       <c r="K30" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L30" s="2" t="n">
         <v>0</v>
@@ -2054,31 +2054,31 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>1.152086744125243</v>
+        <v>1.036478558651414</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>6120</v>
+        <v>5484</v>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>達運</t>
+          <t>慧友</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
         <v/>
       </c>
       <c r="D31" s="2" t="n">
-        <v>361.9346465752073</v>
+        <v>415.6682510653362</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>13.3</v>
+        <v>45.35</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
@@ -2089,13 +2089,13 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>49.41318491417031</v>
+        <v>57.21859493360295</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>16.01910075205851</v>
+        <v>16.69842979840663</v>
       </c>
       <c r="J31" s="2" t="n">
-        <v>0.9138473564552468</v>
+        <v>2.175273072939902</v>
       </c>
       <c r="K31" s="2" t="n">
         <v>0</v>
@@ -2107,31 +2107,31 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>0.1170293593454107</v>
+        <v>0.7378793611678285</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>4960</v>
+        <v>4908</v>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>誠美材</t>
+          <t>前鼎</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
         <v/>
       </c>
       <c r="D32" s="2" t="n">
-        <v>361.1247418044272</v>
+        <v>394.3197722001355</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>20.9</v>
+        <v>155</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
@@ -2142,16 +2142,16 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>42.98995954294531</v>
+        <v>50.16134120066865</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>31.28032771130131</v>
+        <v>24.97686891914095</v>
       </c>
       <c r="J32" s="2" t="n">
-        <v>0.7137574248749289</v>
+        <v>1.114199854340175</v>
       </c>
       <c r="K32" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L32" s="2" t="n">
         <v>0</v>
@@ -2160,7 +2160,7 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>0.4049118445107991</v>
+        <v>4.339458435398978</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
@@ -2170,21 +2170,21 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>4977</v>
+        <v>5228</v>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>眾達-KY</t>
+          <t>鈺鎧</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
         <v/>
       </c>
       <c r="D33" s="2" t="n">
-        <v>357.3125951240739</v>
+        <v>392.5773510079249</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>144.5</v>
+        <v>41.6</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
@@ -2195,16 +2195,16 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>51.88077803988132</v>
+        <v>42.86284189227006</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>22.47005271008175</v>
+        <v>32.23494109930898</v>
       </c>
       <c r="J33" s="2" t="n">
-        <v>1.142811269193213</v>
+        <v>1.241200758689606</v>
       </c>
       <c r="K33" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L33" s="2" t="n">
         <v>0</v>
@@ -2213,31 +2213,31 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>3.891146434182451</v>
+        <v>0.916162958129756</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>5434</v>
+        <v>5236</v>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>崇越</t>
+          <t>凌陽創新</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
         <v/>
       </c>
       <c r="D34" s="2" t="n">
-        <v>354.9211464971661</v>
+        <v>386.1000720665844</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>514</v>
+        <v>144</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
@@ -2248,13 +2248,13 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>49.4262905554853</v>
+        <v>42.52985307112612</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>19.15068386428783</v>
+        <v>32.45358889146563</v>
       </c>
       <c r="J34" s="2" t="n">
-        <v>0.4355403457373043</v>
+        <v>0.4931189176599256</v>
       </c>
       <c r="K34" s="2" t="n">
         <v>0</v>
@@ -2266,31 +2266,31 @@
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>-4.509418653993151</v>
+        <v>0.5890449523042527</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>5292</v>
+        <v>6155</v>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>華懋</t>
+          <t>鈞寶</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
         <v/>
       </c>
       <c r="D35" s="2" t="n">
-        <v>354.8306811316345</v>
+        <v>372.4576796129931</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>178.5</v>
+        <v>53.2</v>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
@@ -2301,13 +2301,13 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>50.88792261330602</v>
+        <v>37.33131055854724</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>28.39246290351197</v>
+        <v>28.61686991395724</v>
       </c>
       <c r="J35" s="2" t="n">
-        <v>0.5053849909022323</v>
+        <v>0.810221052209947</v>
       </c>
       <c r="K35" s="2" t="n">
         <v>0</v>
@@ -2319,48 +2319,48 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>3.399457571870656</v>
+        <v>0.538740303179158</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, adx_trending, obv_uptrend, cci_momentum, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>4908</v>
+        <v>4945</v>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>前鼎</t>
+          <t>陞達科技</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
         <v/>
       </c>
       <c r="D36" s="2" t="n">
-        <v>354.3197722001355</v>
+        <v>371.5300044109481</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>155</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2025-09-01</t>
         </is>
       </c>
       <c r="G36" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>50.16134120066865</v>
+        <v>52.38692800838105</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>24.97686891914095</v>
+        <v>13.93717422322002</v>
       </c>
       <c r="J36" s="2" t="n">
-        <v>1.114199854340175</v>
+        <v>0.4265127663271301</v>
       </c>
       <c r="K36" s="2" t="n">
         <v>2</v>
@@ -2372,31 +2372,31 @@
         <v>-1</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>4.339458435398978</v>
+        <v>0.5968862399752146</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, kd_golden_cross</t>
+          <t>avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>4585</v>
+        <v>4952</v>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>達明</t>
+          <t>凌通</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
         <v/>
       </c>
       <c r="D37" s="2" t="n">
-        <v>349.9203251297397</v>
+        <v>370.8651139957474</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>316</v>
+        <v>49.7</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
@@ -2407,13 +2407,13 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>56.58239988871438</v>
+        <v>49.00483017465969</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>14.60846138224908</v>
+        <v>25.28937153556218</v>
       </c>
       <c r="J37" s="2" t="n">
-        <v>1.34686241012248</v>
+        <v>1.604152488571844</v>
       </c>
       <c r="K37" s="2" t="n">
         <v>0</v>
@@ -2425,31 +2425,31 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>2.939990093150604</v>
+        <v>0.4579933470581394</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>4916</v>
+        <v>5215</v>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>事欣科</t>
+          <t>科嘉-KY</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
         <v/>
       </c>
       <c r="D38" s="2" t="n">
-        <v>346.6986925560279</v>
+        <v>365.4361974913245</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>104</v>
+        <v>38.2</v>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
@@ -2460,13 +2460,13 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>51.38141839917274</v>
+        <v>38.65508097197239</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>15.05931268716882</v>
+        <v>27.13068633506663</v>
       </c>
       <c r="J38" s="2" t="n">
-        <v>1.628099081730125</v>
+        <v>0.2826567577724452</v>
       </c>
       <c r="K38" s="2" t="n">
         <v>0</v>
@@ -2478,31 +2478,31 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>0.7804225735119985</v>
+        <v>0.1298262283225051</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, liquidity_ok, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>6141</v>
+        <v>4949</v>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>柏承</t>
+          <t>有成精密</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
         <v/>
       </c>
       <c r="D39" s="2" t="n">
-        <v>344.3961416574071</v>
+        <v>364.2997256912519</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>34.7</v>
+        <v>72.5</v>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
@@ -2513,13 +2513,13 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>48.45133354773155</v>
+        <v>53.3543493247271</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>14.72794802344577</v>
+        <v>24.48047351854383</v>
       </c>
       <c r="J39" s="2" t="n">
-        <v>0.2575675637235612</v>
+        <v>0.9126413295161788</v>
       </c>
       <c r="K39" s="2" t="n">
         <v>0</v>
@@ -2531,31 +2531,31 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>-0.0719116431093476</v>
+        <v>1.483521275588549</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>4582</v>
+        <v>4577</v>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>聚恆-創</t>
+          <t>達航科技</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
         <v/>
       </c>
       <c r="D40" s="2" t="n">
-        <v>343.3745635687865</v>
+        <v>363.6430796226514</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>28.95</v>
+        <v>78.5</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
@@ -2566,13 +2566,13 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>61.16705129087178</v>
+        <v>50.22445887469512</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>16.8221237140192</v>
+        <v>18.8736438616191</v>
       </c>
       <c r="J40" s="2" t="n">
-        <v>0.9330380709052134</v>
+        <v>0.6892103460494364</v>
       </c>
       <c r="K40" s="2" t="n">
         <v>0</v>
@@ -2584,31 +2584,31 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>0.1409439156349289</v>
+        <v>2.227474854072728</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, liquidity_ok, obv_uptrend, cci_momentum, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>4729</v>
+        <v>4912</v>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>熒茂</t>
+          <t>聯德控股-KY</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
         <v/>
       </c>
       <c r="D41" s="2" t="n">
-        <v>334.2169249182415</v>
+        <v>363.2468637203646</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>20.5</v>
+        <v>89.8</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
@@ -2619,16 +2619,16 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>53.9519710640239</v>
+        <v>56.31566008128947</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>17.01162283010564</v>
+        <v>19.52800831960572</v>
       </c>
       <c r="J41" s="2" t="n">
-        <v>0.8049479162775268</v>
+        <v>1.453387628466162</v>
       </c>
       <c r="K41" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L41" s="2" t="n">
         <v>0</v>
@@ -2637,31 +2637,31 @@
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>0.2954221356026166</v>
+        <v>1.152086744125243</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
-          <t>breakout_20d, market_above_ma60, obv_uptrend, cci_momentum, mfi_strong</t>
+          <t>rsi_strong, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>4906</v>
+        <v>6120</v>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>正文</t>
+          <t>達運</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
         <v/>
       </c>
       <c r="D42" s="2" t="n">
-        <v>325.845273320082</v>
+        <v>361.9346465752073</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>35.6</v>
+        <v>13.3</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
@@ -2672,13 +2672,13 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>48.90227774794005</v>
+        <v>49.41318491417031</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>23.91751543746334</v>
+        <v>16.01910075205851</v>
       </c>
       <c r="J42" s="2" t="n">
-        <v>0.9557856750395342</v>
+        <v>0.9138473564552468</v>
       </c>
       <c r="K42" s="2" t="n">
         <v>0</v>
@@ -2690,31 +2690,31 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>0.5778096343056758</v>
+        <v>0.1170293593454107</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>4577</v>
+        <v>4960</v>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>達航科技</t>
+          <t>誠美材</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
         <v/>
       </c>
       <c r="D43" s="2" t="n">
-        <v>323.6430796226514</v>
+        <v>361.1247418044272</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>78.5</v>
+        <v>20.9</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
@@ -2725,13 +2725,13 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>50.22445887469512</v>
+        <v>42.98995954294531</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>18.8736438616191</v>
+        <v>31.28032771130131</v>
       </c>
       <c r="J43" s="2" t="n">
-        <v>0.6892103460494364</v>
+        <v>0.7137574248749289</v>
       </c>
       <c r="K43" s="2" t="n">
         <v>0</v>
@@ -2743,31 +2743,31 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>2.227474854072728</v>
+        <v>0.4049118445107991</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, liquidity_ok, obv_uptrend, cci_momentum, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>4994</v>
+        <v>4977</v>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>傳奇</t>
+          <t>眾達-KY</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
         <v/>
       </c>
       <c r="D44" s="2" t="n">
-        <v>317.4179188239206</v>
+        <v>357.3125951240739</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>86.90000000000001</v>
+        <v>144.5</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
@@ -2778,13 +2778,13 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>34.99166099349681</v>
+        <v>51.88077803988132</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>20.02648323438446</v>
+        <v>22.47005271008175</v>
       </c>
       <c r="J44" s="2" t="n">
-        <v>0.2914309968708973</v>
+        <v>1.142811269193213</v>
       </c>
       <c r="K44" s="2" t="n">
         <v>0</v>
@@ -2796,31 +2796,31 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>-0.6965345337950284</v>
+        <v>3.891146434182451</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>4934</v>
+        <v>5434</v>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>太極</t>
+          <t>崇越</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
         <v/>
       </c>
       <c r="D45" s="2" t="n">
-        <v>315.5927305427393</v>
+        <v>354.9211464971661</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>14.35</v>
+        <v>514</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
@@ -2831,13 +2831,13 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>41.30553182405843</v>
+        <v>49.4262905554853</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>23.13699298382795</v>
+        <v>19.15068386428783</v>
       </c>
       <c r="J45" s="2" t="n">
-        <v>0.6834227693278496</v>
+        <v>0.4355403457373043</v>
       </c>
       <c r="K45" s="2" t="n">
         <v>0</v>
@@ -2849,31 +2849,31 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>0.0341253836370308</v>
+        <v>-4.509418653993151</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>6115</v>
+        <v>5292</v>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>鎰勝</t>
+          <t>華懋</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
         <v/>
       </c>
       <c r="D46" s="2" t="n">
-        <v>310.2074539838557</v>
+        <v>354.8306811316345</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>45.25</v>
+        <v>178.5</v>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
@@ -2884,13 +2884,13 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>40.31672645177468</v>
+        <v>50.88792261330602</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>21.714296571618</v>
+        <v>28.39246290351197</v>
       </c>
       <c r="J46" s="2" t="n">
-        <v>0.5061587967026387</v>
+        <v>0.5053849909022323</v>
       </c>
       <c r="K46" s="2" t="n">
         <v>0</v>
@@ -2902,31 +2902,31 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>0.0415849828505581</v>
+        <v>3.399457571870656</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
+          <t>market_above_ma60, adx_trending, obv_uptrend, cci_momentum, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>5258</v>
+        <v>4585</v>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>虹堡</t>
+          <t>達明</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
         <v/>
       </c>
       <c r="D47" s="2" t="n">
-        <v>306.39010904938</v>
+        <v>349.9203251297397</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>53.2</v>
+        <v>316</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
@@ -2937,13 +2937,13 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>53.78560276215403</v>
+        <v>56.58239988871438</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>10.95366914599148</v>
+        <v>14.60846138224908</v>
       </c>
       <c r="J47" s="2" t="n">
-        <v>0.7941218939081219</v>
+        <v>1.34686241012248</v>
       </c>
       <c r="K47" s="2" t="n">
         <v>0</v>
@@ -2955,31 +2955,31 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>0.0595228754811225</v>
+        <v>2.939990093150604</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend</t>
+          <t>rsi_strong, market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>4554</v>
+        <v>4916</v>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>橙的</t>
+          <t>事欣科</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
         <v/>
       </c>
       <c r="D48" s="2" t="n">
-        <v>297.5191354372515</v>
+        <v>346.6986925560279</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>31</v>
+        <v>104</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
@@ -2990,13 +2990,13 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>52.81480341396858</v>
+        <v>51.38141839917274</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>16.21632272689332</v>
+        <v>15.05931268716882</v>
       </c>
       <c r="J48" s="2" t="n">
-        <v>0.3514974901685374</v>
+        <v>1.628099081730125</v>
       </c>
       <c r="K48" s="2" t="n">
         <v>0</v>
@@ -3008,31 +3008,31 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>0.0288193677908936</v>
+        <v>0.7804225735119985</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, avoid_chase, hist_turn_positive</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>5244</v>
+        <v>6141</v>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>弘凱</t>
+          <t>柏承</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
         <v/>
       </c>
       <c r="D49" s="2" t="n">
-        <v>296.8660303529277</v>
+        <v>344.3961416574071</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>33.45</v>
+        <v>34.7</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
@@ -3043,13 +3043,13 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>53.30223996170341</v>
+        <v>48.45133354773155</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>30.52603777036415</v>
+        <v>14.72794802344577</v>
       </c>
       <c r="J49" s="2" t="n">
-        <v>0.3143485472156205</v>
+        <v>0.2575675637235612</v>
       </c>
       <c r="K49" s="2" t="n">
         <v>0</v>
@@ -3061,31 +3061,31 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>0.5165268561921237</v>
+        <v>-0.0719116431093476</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>5243</v>
+        <v>4582</v>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>乙盛-KY</t>
+          <t>聚恆-創</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
         <v/>
       </c>
       <c r="D50" s="2" t="n">
-        <v>292.8689566686492</v>
+        <v>343.3745635687865</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>88.7</v>
+        <v>28.95</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -3096,13 +3096,13 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>48.91911065206893</v>
+        <v>61.16705129087178</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>26.85436890317077</v>
+        <v>16.8221237140192</v>
       </c>
       <c r="J50" s="2" t="n">
-        <v>0.8201845322182026</v>
+        <v>0.9330380709052134</v>
       </c>
       <c r="K50" s="2" t="n">
         <v>0</v>
@@ -3114,31 +3114,31 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>1.507139789455743</v>
+        <v>0.1409439156349289</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>5285</v>
+        <v>4554</v>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>界霖</t>
+          <t>橙的</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
         <v/>
       </c>
       <c r="D51" s="2" t="n">
-        <v>292.4666434513362</v>
+        <v>337.5191354372515</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>77.90000000000001</v>
+        <v>31</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
@@ -3149,13 +3149,13 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>46.03131847409194</v>
+        <v>52.81480341396858</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>26.25728421109625</v>
+        <v>16.21632272689332</v>
       </c>
       <c r="J51" s="2" t="n">
-        <v>0.7783736006083323</v>
+        <v>0.3514974901685374</v>
       </c>
       <c r="K51" s="2" t="n">
         <v>0</v>
@@ -3167,31 +3167,31 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>0.6016897874066061</v>
+        <v>0.0288193677908936</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending</t>
+          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, avoid_chase, hist_turn_positive</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>5234</v>
+        <v>4729</v>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>達興材料</t>
+          <t>熒茂</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
         <v/>
       </c>
       <c r="D52" s="2" t="n">
-        <v>285.7503582925585</v>
+        <v>334.2169249182415</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>333</v>
+        <v>20.5</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
@@ -3202,16 +3202,16 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>45.76404322672544</v>
+        <v>53.9519710640239</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>33.48991363390045</v>
+        <v>17.01162283010564</v>
       </c>
       <c r="J52" s="2" t="n">
-        <v>0.3586877010511765</v>
+        <v>0.8049479162775268</v>
       </c>
       <c r="K52" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L52" s="2" t="n">
         <v>0</v>
@@ -3220,31 +3220,31 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>3.369837355019246</v>
+        <v>0.2954221356026166</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>breakout_20d, market_above_ma60, obv_uptrend, cci_momentum, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>5225</v>
+        <v>4906</v>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>東科-KY</t>
+          <t>正文</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
         <v/>
       </c>
       <c r="D53" s="2" t="n">
-        <v>280.932078295633</v>
+        <v>325.845273320082</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>66.7</v>
+        <v>35.6</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
@@ -3255,13 +3255,13 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>34.14449300849357</v>
+        <v>48.90227774794005</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>17.18448703150719</v>
+        <v>23.91751543746334</v>
       </c>
       <c r="J53" s="2" t="n">
-        <v>5.808678706514208</v>
+        <v>0.9557856750395342</v>
       </c>
       <c r="K53" s="2" t="n">
         <v>0</v>
@@ -3273,31 +3273,31 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>-0.1504005653047247</v>
+        <v>0.5778096343056758</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>4905</v>
+        <v>4994</v>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>台聯電</t>
+          <t>傳奇</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
         <v/>
       </c>
       <c r="D54" s="2" t="n">
-        <v>276.8105776637935</v>
+        <v>317.4179188239206</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>68.2</v>
+        <v>86.90000000000001</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>52.04194454984401</v>
+        <v>34.99166099349681</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>7.319445248533803</v>
+        <v>20.02648323438446</v>
       </c>
       <c r="J54" s="2" t="n">
-        <v>1.26740453260505</v>
+        <v>0.2914309968708973</v>
       </c>
       <c r="K54" s="2" t="n">
         <v>0</v>
@@ -3326,31 +3326,31 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>1.233821332386999</v>
+        <v>-0.6965345337950284</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>4545</v>
+        <v>4905</v>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>銘鈺</t>
+          <t>台聯電</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
         <v/>
       </c>
       <c r="D55" s="2" t="n">
-        <v>273.7702291199062</v>
+        <v>316.8105776637935</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>33</v>
+        <v>68.2</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
@@ -3361,13 +3361,13 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>44.91578159532225</v>
+        <v>52.04194454984401</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>23.35628152857437</v>
+        <v>7.319445248533803</v>
       </c>
       <c r="J55" s="2" t="n">
-        <v>0.5393053711060163</v>
+        <v>1.26740453260505</v>
       </c>
       <c r="K55" s="2" t="n">
         <v>0</v>
@@ -3379,31 +3379,31 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>0.1233672252941779</v>
+        <v>1.233821332386999</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>4904</v>
+        <v>4934</v>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>遠傳</t>
+          <t>太極</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
         <v/>
       </c>
       <c r="D56" s="2" t="n">
-        <v>271.2312401535603</v>
+        <v>315.5927305427393</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>101.5</v>
+        <v>14.35</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
@@ -3414,13 +3414,13 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>46.55732622350491</v>
+        <v>41.30553182405843</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>16.29740275134491</v>
+        <v>23.13699298382795</v>
       </c>
       <c r="J56" s="2" t="n">
-        <v>0.2833510144202986</v>
+        <v>0.6834227693278496</v>
       </c>
       <c r="K56" s="2" t="n">
         <v>0</v>
@@ -3432,31 +3432,31 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>-0.2794630996128649</v>
+        <v>0.0341253836370308</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>4958</v>
+        <v>4972</v>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>臻鼎-KY</t>
+          <t>湯石照明</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
         <v/>
       </c>
       <c r="D57" s="2" t="n">
-        <v>261.4785485577389</v>
+        <v>312.4836601882047</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>470.5</v>
+        <v>16.6</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
@@ -3467,13 +3467,13 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>46.37462581364231</v>
+        <v>47.3412259077718</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>20.3110168592201</v>
+        <v>23.38176882618041</v>
       </c>
       <c r="J57" s="2" t="n">
-        <v>0.8578887123864128</v>
+        <v>0.8501235460147865</v>
       </c>
       <c r="K57" s="2" t="n">
         <v>0</v>
@@ -3485,31 +3485,31 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>2.955173099935717</v>
+        <v>-0.0025725966735486</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>4968</v>
+        <v>6115</v>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>立積</t>
+          <t>鎰勝</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
         <v/>
       </c>
       <c r="D58" s="2" t="n">
-        <v>261.2839316525766</v>
+        <v>310.2074539838557</v>
       </c>
       <c r="E58" s="2" t="n">
-        <v>96</v>
+        <v>45.25</v>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
@@ -3520,13 +3520,13 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>42.6023614203129</v>
+        <v>40.31672645177468</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>29.2589159880538</v>
+        <v>21.714296571618</v>
       </c>
       <c r="J58" s="2" t="n">
-        <v>0.5314670321843064</v>
+        <v>0.5061587967026387</v>
       </c>
       <c r="K58" s="2" t="n">
         <v>0</v>
@@ -3538,31 +3538,31 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>0.5574478353948109</v>
+        <v>0.0415849828505581</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>6139</v>
+        <v>5258</v>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>亞翔</t>
+          <t>虹堡</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
         <v/>
       </c>
       <c r="D59" s="2" t="n">
-        <v>261.0775800347633</v>
+        <v>306.39010904938</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>808</v>
+        <v>53.2</v>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
@@ -3573,13 +3573,13 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>51.04780791299308</v>
+        <v>53.78560276215403</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>16.36860798565198</v>
+        <v>10.95366914599148</v>
       </c>
       <c r="J59" s="2" t="n">
-        <v>0.8699903491719368</v>
+        <v>0.7941218939081219</v>
       </c>
       <c r="K59" s="2" t="n">
         <v>0</v>
@@ -3591,31 +3591,31 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>6.488097113718801</v>
+        <v>0.0595228754811225</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>4956</v>
+        <v>5244</v>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>光鋐</t>
+          <t>弘凱</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
         <v/>
       </c>
       <c r="D60" s="2" t="n">
-        <v>259.1290759239308</v>
+        <v>296.8660303529277</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>31.4</v>
+        <v>33.45</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
@@ -3626,13 +3626,13 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>49.00296475184222</v>
+        <v>53.30223996170341</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>22.28994792980012</v>
+        <v>30.52603777036415</v>
       </c>
       <c r="J60" s="2" t="n">
-        <v>1.090149792074088</v>
+        <v>0.3143485472156205</v>
       </c>
       <c r="K60" s="2" t="n">
         <v>0</v>
@@ -3644,31 +3644,31 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>0.818659712514306</v>
+        <v>0.5165268561921237</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, adx_trending, mfi_strong</t>
+          <t>market_above_ma60, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>4749</v>
+        <v>5220</v>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>新應材</t>
+          <t>萬達光電</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
         <v/>
       </c>
       <c r="D61" s="2" t="n">
-        <v>252.4553970786563</v>
+        <v>296.006239060267</v>
       </c>
       <c r="E61" s="2" t="n">
-        <v>786</v>
+        <v>20.5</v>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
@@ -3679,16 +3679,16 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>45.85009892542204</v>
+        <v>45.8224167425146</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>24.86203343788427</v>
+        <v>19.80084211670331</v>
       </c>
       <c r="J61" s="2" t="n">
-        <v>1.331690192582099</v>
+        <v>1.420440721559904</v>
       </c>
       <c r="K61" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L61" s="2" t="n">
         <v>0</v>
@@ -3697,31 +3697,31 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>12.25410963376711</v>
+        <v>0.0297183915284491</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>4927</v>
+        <v>5227</v>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>泰鼎-KY</t>
+          <t>立凱-KY</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
         <v/>
       </c>
       <c r="D62" s="2" t="n">
-        <v>248.2292252295517</v>
+        <v>293.2876398456008</v>
       </c>
       <c r="E62" s="2" t="n">
-        <v>33.8</v>
+        <v>34</v>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
@@ -3732,13 +3732,13 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>43.86216628911887</v>
+        <v>46.83097606435219</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>37.46306240323691</v>
+        <v>15.56843498902705</v>
       </c>
       <c r="J62" s="2" t="n">
-        <v>0.9302535541838</v>
+        <v>0.5344587708073099</v>
       </c>
       <c r="K62" s="2" t="n">
         <v>0</v>
@@ -3750,31 +3750,31 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>0.7539762670325443</v>
+        <v>-0.624716331617889</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, liquidity_ok, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, kd_golden_cross, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>4909</v>
+        <v>5243</v>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>新復興</t>
+          <t>乙盛-KY</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
         <v/>
       </c>
       <c r="D63" s="2" t="n">
-        <v>218.7844530833949</v>
+        <v>292.8689566686492</v>
       </c>
       <c r="E63" s="2" t="n">
-        <v>38.65</v>
+        <v>88.7</v>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
@@ -3785,13 +3785,13 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>45.18805287593229</v>
+        <v>48.91911065206893</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>45.1175850381016</v>
+        <v>26.85436890317077</v>
       </c>
       <c r="J63" s="2" t="n">
-        <v>0.5339147467393848</v>
+        <v>0.8201845322182026</v>
       </c>
       <c r="K63" s="2" t="n">
         <v>0</v>
@@ -3803,31 +3803,31 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>0.5930819272115464</v>
+        <v>1.507139789455743</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, adx_trending, dealer_buy_3d</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>6133</v>
+        <v>5285</v>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>金橋</t>
+          <t>界霖</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
         <v/>
       </c>
       <c r="D64" s="2" t="n">
-        <v>216.5540279577056</v>
+        <v>292.4666434513362</v>
       </c>
       <c r="E64" s="2" t="n">
-        <v>21.65</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
@@ -3838,13 +3838,13 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>50.20113041156037</v>
+        <v>46.03131847409194</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>20.28018297898767</v>
+        <v>26.25728421109625</v>
       </c>
       <c r="J64" s="2" t="n">
-        <v>0.7411851229408724</v>
+        <v>0.7783736006083323</v>
       </c>
       <c r="K64" s="2" t="n">
         <v>0</v>
@@ -3856,31 +3856,31 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>0.199736224925178</v>
+        <v>0.6016897874066061</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>6128</v>
+        <v>4749</v>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>上福</t>
+          <t>新應材</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
         <v/>
       </c>
       <c r="D65" s="2" t="n">
-        <v>207.0924510619332</v>
+        <v>292.4553970786563</v>
       </c>
       <c r="E65" s="2" t="n">
-        <v>20.25</v>
+        <v>786</v>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
@@ -3891,13 +3891,13 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>49.9826959025004</v>
+        <v>45.85009892542204</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>11.37570190222946</v>
+        <v>24.86203343788427</v>
       </c>
       <c r="J65" s="2" t="n">
-        <v>0.6315679802937335</v>
+        <v>1.331690192582099</v>
       </c>
       <c r="K65" s="2" t="n">
         <v>0</v>
@@ -3909,31 +3909,31 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>-0.0016259974820021</v>
+        <v>12.25410963376711</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>4943</v>
+        <v>5234</v>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>康控-KY</t>
+          <t>達興材料</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
         <v/>
       </c>
       <c r="D66" s="2" t="n">
-        <v>206.1136396113312</v>
+        <v>285.7503582925585</v>
       </c>
       <c r="E66" s="2" t="n">
-        <v>8.73</v>
+        <v>333</v>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
@@ -3944,13 +3944,13 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>49.83733034863605</v>
+        <v>45.76404322672544</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>10.86796595360301</v>
+        <v>33.48991363390045</v>
       </c>
       <c r="J66" s="2" t="n">
-        <v>2.157778526767597</v>
+        <v>0.3586877010511765</v>
       </c>
       <c r="K66" s="2" t="n">
         <v>0</v>
@@ -3962,31 +3962,31 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>0.0213091663164116</v>
+        <v>3.369837355019246</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>4588</v>
+        <v>4966</v>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>玖鼎電力</t>
+          <t>譜瑞-KY</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
         <v/>
       </c>
       <c r="D67" s="2" t="n">
-        <v>200.4183031855675</v>
+        <v>285.2089964925678</v>
       </c>
       <c r="E67" s="2" t="n">
-        <v>52.3</v>
+        <v>600</v>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
@@ -3997,49 +3997,49 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>46.71206210564022</v>
+        <v>47.73446130319673</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>11.74067879935242</v>
+        <v>24.29655162171155</v>
       </c>
       <c r="J67" s="2" t="n">
-        <v>0.7120002173535946</v>
+        <v>0.6734724378048407</v>
       </c>
       <c r="K67" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L67" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M67" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>0.3367779917088633</v>
+        <v>5.538093920247391</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>6117</v>
+        <v>5225</v>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>迎廣</t>
+          <t>東科-KY</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
         <v/>
       </c>
       <c r="D68" s="2" t="n">
-        <v>175.2160314232809</v>
+        <v>280.932078295633</v>
       </c>
       <c r="E68" s="2" t="n">
-        <v>66.3</v>
+        <v>66.7</v>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
@@ -4050,13 +4050,13 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>43.13001193649077</v>
+        <v>34.14449300849357</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>35.39311846332311</v>
+        <v>17.18448703150719</v>
       </c>
       <c r="J68" s="2" t="n">
-        <v>0.5350356520416067</v>
+        <v>5.808678706514208</v>
       </c>
       <c r="K68" s="2" t="n">
         <v>0</v>
@@ -4068,31 +4068,31 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>0.429867101486832</v>
+        <v>-0.1504005653047247</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>volume_break, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>4935</v>
+        <v>4545</v>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>茂林-KY</t>
+          <t>銘鈺</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
         <v/>
       </c>
       <c r="D69" s="2" t="n">
-        <v>162.8516923869098</v>
+        <v>273.7702291199062</v>
       </c>
       <c r="E69" s="2" t="n">
-        <v>34.9</v>
+        <v>33</v>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
@@ -4103,13 +4103,13 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>44.24872811142037</v>
+        <v>44.91578159532225</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>25.22631528415401</v>
+        <v>23.35628152857437</v>
       </c>
       <c r="J69" s="2" t="n">
-        <v>0.4113438878876249</v>
+        <v>0.5393053711060163</v>
       </c>
       <c r="K69" s="2" t="n">
         <v>0</v>
@@ -4121,31 +4121,31 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>0.0719990356201272</v>
+        <v>0.1233672252941779</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>4942</v>
+        <v>4904</v>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>嘉彰</t>
+          <t>遠傳</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
         <v/>
       </c>
       <c r="D70" s="2" t="n">
-        <v>149.1782224943766</v>
+        <v>271.2312401535603</v>
       </c>
       <c r="E70" s="2" t="n">
-        <v>34.4</v>
+        <v>101.5</v>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
@@ -4156,13 +4156,13 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>32.71435058313217</v>
+        <v>46.55732622350491</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>34.7439689552841</v>
+        <v>16.29740275134491</v>
       </c>
       <c r="J70" s="2" t="n">
-        <v>0.1479934475324105</v>
+        <v>0.2833510144202986</v>
       </c>
       <c r="K70" s="2" t="n">
         <v>0</v>
@@ -4174,31 +4174,31 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>-0.1351670077672591</v>
+        <v>-0.2794630996128649</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>5203</v>
+        <v>4958</v>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>訊連</t>
+          <t>臻鼎-KY</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
         <v/>
       </c>
       <c r="D71" s="2" t="n">
-        <v>101.9737429417021</v>
+        <v>261.4785485577389</v>
       </c>
       <c r="E71" s="2" t="n">
-        <v>66.3</v>
+        <v>470.5</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
@@ -4209,13 +4209,13 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>49.56727574013343</v>
+        <v>46.37462581364231</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>13.13222341744633</v>
+        <v>20.3110168592201</v>
       </c>
       <c r="J71" s="2" t="n">
-        <v>0.9995970540724868</v>
+        <v>0.8578887123864128</v>
       </c>
       <c r="K71" s="2" t="n">
         <v>0</v>
@@ -4227,62 +4227,1069 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>0.2019787610738842</v>
+        <v>2.955173099935717</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
+        <v>4968</v>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>立積</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D72" s="2" t="n">
+        <v>261.2839316525766</v>
+      </c>
+      <c r="E72" s="2" t="n">
+        <v>96</v>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H72" s="2" t="n">
+        <v>42.6023614203129</v>
+      </c>
+      <c r="I72" s="2" t="n">
+        <v>29.2589159880538</v>
+      </c>
+      <c r="J72" s="2" t="n">
+        <v>0.5314670321843064</v>
+      </c>
+      <c r="K72" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L72" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M72" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N72" s="2" t="n">
+        <v>0.5574478353948109</v>
+      </c>
+      <c r="O72" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>6139</v>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>亞翔</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D73" s="2" t="n">
+        <v>261.0775800347633</v>
+      </c>
+      <c r="E73" s="2" t="n">
+        <v>808</v>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H73" s="2" t="n">
+        <v>51.04780791299308</v>
+      </c>
+      <c r="I73" s="2" t="n">
+        <v>16.36860798565198</v>
+      </c>
+      <c r="J73" s="2" t="n">
+        <v>0.8699903491719368</v>
+      </c>
+      <c r="K73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M73" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N73" s="2" t="n">
+        <v>6.488097113718801</v>
+      </c>
+      <c r="O73" s="2" t="inlineStr">
+        <is>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, mfi_strong</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>4956</v>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>光鋐</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D74" s="2" t="n">
+        <v>259.1290759239308</v>
+      </c>
+      <c r="E74" s="2" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H74" s="2" t="n">
+        <v>49.00296475184222</v>
+      </c>
+      <c r="I74" s="2" t="n">
+        <v>22.28994792980012</v>
+      </c>
+      <c r="J74" s="2" t="n">
+        <v>1.090149792074088</v>
+      </c>
+      <c r="K74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M74" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N74" s="2" t="n">
+        <v>0.818659712514306</v>
+      </c>
+      <c r="O74" s="2" t="inlineStr">
+        <is>
+          <t>ema60_gt_ema120, market_above_ma60, adx_trending, mfi_strong</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>4927</v>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>泰鼎-KY</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D75" s="2" t="n">
+        <v>248.2292252295517</v>
+      </c>
+      <c r="E75" s="2" t="n">
+        <v>33.8</v>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H75" s="2" t="n">
+        <v>43.86216628911887</v>
+      </c>
+      <c r="I75" s="2" t="n">
+        <v>37.46306240323691</v>
+      </c>
+      <c r="J75" s="2" t="n">
+        <v>0.9302535541838</v>
+      </c>
+      <c r="K75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M75" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N75" s="2" t="n">
+        <v>0.7539762670325443</v>
+      </c>
+      <c r="O75" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, liquidity_ok, adx_trending</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>4974</v>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>亞泰</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D76" s="2" t="n">
+        <v>240.7559572902474</v>
+      </c>
+      <c r="E76" s="2" t="n">
+        <v>69.7</v>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H76" s="2" t="n">
+        <v>53.77588547359791</v>
+      </c>
+      <c r="I76" s="2" t="n">
+        <v>19.9779382479398</v>
+      </c>
+      <c r="J76" s="2" t="n">
+        <v>0.5571673518292809</v>
+      </c>
+      <c r="K76" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="L76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M76" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N76" s="2" t="n">
+        <v>0.4545185342767697</v>
+      </c>
+      <c r="O76" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>4923</v>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>力士</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D77" s="2" t="n">
+        <v>234.7800600060681</v>
+      </c>
+      <c r="E77" s="2" t="n">
+        <v>49.85</v>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H77" s="2" t="n">
+        <v>53.98713054906118</v>
+      </c>
+      <c r="I77" s="2" t="n">
+        <v>21.96572354246468</v>
+      </c>
+      <c r="J77" s="2" t="n">
+        <v>0.5509997120283362</v>
+      </c>
+      <c r="K77" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="L77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M77" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N77" s="2" t="n">
+        <v>0.6419361873166363</v>
+      </c>
+      <c r="O77" s="2" t="inlineStr">
+        <is>
+          <t>ema60_gt_ema120, market_above_ma60, adx_trending</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>6133</v>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>金橋</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D78" s="2" t="n">
+        <v>216.5540279577056</v>
+      </c>
+      <c r="E78" s="2" t="n">
+        <v>21.65</v>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H78" s="2" t="n">
+        <v>50.20113041156037</v>
+      </c>
+      <c r="I78" s="2" t="n">
+        <v>20.28018297898767</v>
+      </c>
+      <c r="J78" s="2" t="n">
+        <v>0.7411851229408724</v>
+      </c>
+      <c r="K78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M78" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N78" s="2" t="n">
+        <v>0.199736224925178</v>
+      </c>
+      <c r="O78" s="2" t="inlineStr">
+        <is>
+          <t>ema60_gt_ema120, market_above_ma60, adx_trending</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>5223</v>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>安力-KY</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D79" s="2" t="n">
+        <v>210.6301540387188</v>
+      </c>
+      <c r="E79" s="2" t="n">
+        <v>23.75</v>
+      </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H79" s="2" t="n">
+        <v>51.51340845832883</v>
+      </c>
+      <c r="I79" s="2" t="n">
+        <v>34.73510475654897</v>
+      </c>
+      <c r="J79" s="2" t="n">
+        <v>0.6358218277633472</v>
+      </c>
+      <c r="K79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M79" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N79" s="2" t="n">
+        <v>0.1371766551739001</v>
+      </c>
+      <c r="O79" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>4933</v>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>友輝</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D80" s="2" t="n">
+        <v>207.2712433341504</v>
+      </c>
+      <c r="E80" s="2" t="n">
+        <v>55.1</v>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H80" s="2" t="n">
+        <v>39.04774732321111</v>
+      </c>
+      <c r="I80" s="2" t="n">
+        <v>32.04593950688626</v>
+      </c>
+      <c r="J80" s="2" t="n">
+        <v>1.356180031055279</v>
+      </c>
+      <c r="K80" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="L80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M80" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N80" s="2" t="n">
+        <v>0.4553502097314617</v>
+      </c>
+      <c r="O80" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>6128</v>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>上福</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D81" s="2" t="n">
+        <v>207.0924510619332</v>
+      </c>
+      <c r="E81" s="2" t="n">
+        <v>20.25</v>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H81" s="2" t="n">
+        <v>49.9826959025004</v>
+      </c>
+      <c r="I81" s="2" t="n">
+        <v>11.37570190222946</v>
+      </c>
+      <c r="J81" s="2" t="n">
+        <v>0.6315679802937335</v>
+      </c>
+      <c r="K81" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L81" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M81" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N81" s="2" t="n">
+        <v>-0.0016259974820021</v>
+      </c>
+      <c r="O81" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>4943</v>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>康控-KY</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D82" s="2" t="n">
+        <v>206.1136396113312</v>
+      </c>
+      <c r="E82" s="2" t="n">
+        <v>8.73</v>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H82" s="2" t="n">
+        <v>49.83733034863605</v>
+      </c>
+      <c r="I82" s="2" t="n">
+        <v>10.86796595360301</v>
+      </c>
+      <c r="J82" s="2" t="n">
+        <v>2.157778526767597</v>
+      </c>
+      <c r="K82" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L82" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M82" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N82" s="2" t="n">
+        <v>0.0213091663164116</v>
+      </c>
+      <c r="O82" s="2" t="inlineStr">
+        <is>
+          <t>volume_break, market_above_ma60, avoid_chase</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>4588</v>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>玖鼎電力</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D83" s="2" t="n">
+        <v>200.4183031855675</v>
+      </c>
+      <c r="E83" s="2" t="n">
+        <v>52.3</v>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H83" s="2" t="n">
+        <v>46.71206210564022</v>
+      </c>
+      <c r="I83" s="2" t="n">
+        <v>11.74067879935242</v>
+      </c>
+      <c r="J83" s="2" t="n">
+        <v>0.7120002173535946</v>
+      </c>
+      <c r="K83" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L83" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M83" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N83" s="2" t="n">
+        <v>0.3367779917088633</v>
+      </c>
+      <c r="O83" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase, mfi_strong</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>4909</v>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>新復興</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D84" s="2" t="n">
+        <v>188.7844530833949</v>
+      </c>
+      <c r="E84" s="2" t="n">
+        <v>38.65</v>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H84" s="2" t="n">
+        <v>45.18805287593229</v>
+      </c>
+      <c r="I84" s="2" t="n">
+        <v>45.1175850381016</v>
+      </c>
+      <c r="J84" s="2" t="n">
+        <v>0.5339147467393848</v>
+      </c>
+      <c r="K84" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L84" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M84" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N84" s="2" t="n">
+        <v>0.5930819272115464</v>
+      </c>
+      <c r="O84" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, adx_trending, dealer_buy_3d</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>5205</v>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>中茂</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D85" s="2" t="n">
+        <v>180.7344639414117</v>
+      </c>
+      <c r="E85" s="2" t="n">
+        <v>21.85</v>
+      </c>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H85" s="2" t="n">
+        <v>49.65510841223037</v>
+      </c>
+      <c r="I85" s="2" t="n">
+        <v>16.22261013389423</v>
+      </c>
+      <c r="J85" s="2" t="n">
+        <v>2.12401055408971</v>
+      </c>
+      <c r="K85" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L85" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M85" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N85" s="2" t="n">
+        <v>0.1014608900464688</v>
+      </c>
+      <c r="O85" s="2" t="inlineStr">
+        <is>
+          <t>volume_break, market_above_ma60, avoid_chase</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>6117</v>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>迎廣</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D86" s="2" t="n">
+        <v>175.2160314232809</v>
+      </c>
+      <c r="E86" s="2" t="n">
+        <v>66.3</v>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G86" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H86" s="2" t="n">
+        <v>43.13001193649077</v>
+      </c>
+      <c r="I86" s="2" t="n">
+        <v>35.39311846332311</v>
+      </c>
+      <c r="J86" s="2" t="n">
+        <v>0.5350356520416067</v>
+      </c>
+      <c r="K86" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L86" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M86" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N86" s="2" t="n">
+        <v>0.429867101486832</v>
+      </c>
+      <c r="O86" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>4935</v>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>茂林-KY</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D87" s="2" t="n">
+        <v>162.8516923869098</v>
+      </c>
+      <c r="E87" s="2" t="n">
+        <v>34.9</v>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H87" s="2" t="n">
+        <v>44.24872811142037</v>
+      </c>
+      <c r="I87" s="2" t="n">
+        <v>25.22631528415401</v>
+      </c>
+      <c r="J87" s="2" t="n">
+        <v>0.4113438878876249</v>
+      </c>
+      <c r="K87" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L87" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M87" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N87" s="2" t="n">
+        <v>0.0719990356201272</v>
+      </c>
+      <c r="O87" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>4924</v>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>欣厚-KY</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D88" s="2" t="n">
+        <v>154.6535142617076</v>
+      </c>
+      <c r="E88" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H88" s="2" t="n">
+        <v>40.88872154161214</v>
+      </c>
+      <c r="I88" s="2" t="n">
+        <v>15.24132756065156</v>
+      </c>
+      <c r="J88" s="2" t="n">
+        <v>0.3628182009187222</v>
+      </c>
+      <c r="K88" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L88" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M88" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N88" s="2" t="n">
+        <v>0.0913781522050604</v>
+      </c>
+      <c r="O88" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>4942</v>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>嘉彰</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D89" s="2" t="n">
+        <v>149.1782224943766</v>
+      </c>
+      <c r="E89" s="2" t="n">
+        <v>34.4</v>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H89" s="2" t="n">
+        <v>32.71435058313217</v>
+      </c>
+      <c r="I89" s="2" t="n">
+        <v>34.7439689552841</v>
+      </c>
+      <c r="J89" s="2" t="n">
+        <v>0.1479934475324105</v>
+      </c>
+      <c r="K89" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L89" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M89" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N89" s="2" t="n">
+        <v>-0.1351670077672591</v>
+      </c>
+      <c r="O89" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>5203</v>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>訊連</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D90" s="2" t="n">
+        <v>101.9737429417021</v>
+      </c>
+      <c r="E90" s="2" t="n">
+        <v>66.3</v>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H90" s="2" t="n">
+        <v>49.56727574013343</v>
+      </c>
+      <c r="I90" s="2" t="n">
+        <v>13.13222341744633</v>
+      </c>
+      <c r="J90" s="2" t="n">
+        <v>0.9995970540724868</v>
+      </c>
+      <c r="K90" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L90" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M90" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N90" s="2" t="n">
+        <v>0.2019787610738842</v>
+      </c>
+      <c r="O90" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
         <v>5222</v>
       </c>
-      <c r="B72" s="2" t="inlineStr">
+      <c r="B91" s="2" t="inlineStr">
         <is>
           <t>全訊</t>
         </is>
       </c>
-      <c r="C72" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D72" s="2" t="n">
+      <c r="C91" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D91" s="2" t="n">
         <v>22.57427690845608</v>
       </c>
-      <c r="E72" s="2" t="n">
+      <c r="E91" s="2" t="n">
         <v>117</v>
       </c>
-      <c r="F72" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
-        </is>
-      </c>
-      <c r="G72" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H72" s="2" t="n">
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H91" s="2" t="n">
         <v>52.13988548325485</v>
       </c>
-      <c r="I72" s="2" t="n">
+      <c r="I91" s="2" t="n">
         <v>15.2842624705879</v>
       </c>
-      <c r="J72" s="2" t="n">
+      <c r="J91" s="2" t="n">
         <v>0.7069510284207264</v>
       </c>
-      <c r="K72" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L72" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M72" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="N72" s="2" t="n">
+      <c r="K91" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L91" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M91" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N91" s="2" t="n">
         <v>0.5065730557108097</v>
       </c>
-      <c r="O72" s="2" t="inlineStr">
+      <c r="O91" s="2" t="inlineStr">
         <is>
           <t>market_above_ma60</t>
         </is>

</xml_diff>